<commit_message>
Output of cv and rechnung improved
</commit_message>
<xml_diff>
--- a/data/rechnung/Rechnungsbeträge.xlsx
+++ b/data/rechnung/Rechnungsbeträge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frank\git\document-generator\data\rechnung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5297E8CB-E66F-45A8-A455-AA2307E17664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C649762E-30EA-490B-AE9B-4403274A6F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40560" yWindow="4320" windowWidth="28800" windowHeight="15345" xr2:uid="{79AF68BE-ECC0-4E6F-85E2-599950CEF42A}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>Preis</t>
   </si>
   <si>
-    <t>Testmanagement</t>
-  </si>
-  <si>
     <t>Projektmanagement</t>
   </si>
   <si>
@@ -72,6 +69,10 @@
   </si>
   <si>
     <t>Dauer [h]</t>
+  </si>
+  <si>
+    <t>Testmanagement
+einschl. Testreporting</t>
   </si>
 </sst>
 </file>
@@ -81,7 +82,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,7 +92,13 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -99,10 +106,11 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -381,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
@@ -394,35 +402,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -757,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73334B3D-398F-4D65-A8B1-8258F9625DBC}">
-  <dimension ref="B2:H16"/>
+  <dimension ref="B2:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
@@ -776,13 +785,13 @@
       <c r="G2" s="3"/>
       <c r="H2" s="5"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6"/>
       <c r="C3" s="12" t="s">
         <v>0</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>1</v>
@@ -795,170 +804,125 @@
       </c>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" ht="27" x14ac:dyDescent="0.25">
       <c r="B4" s="6"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="15"/>
+      <c r="C4" s="14">
+        <v>46255</v>
+      </c>
+      <c r="D4" s="15">
+        <v>8.5</v>
+      </c>
+      <c r="E4" s="16">
+        <v>1500</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="18">
+        <f>D4*E4</f>
+        <v>12750</v>
+      </c>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="6"/>
-      <c r="C5" s="16">
-        <v>46255</v>
-      </c>
-      <c r="D5" s="17">
-        <v>8.5</v>
-      </c>
-      <c r="E5" s="18">
+      <c r="C5" s="19">
+        <v>46256</v>
+      </c>
+      <c r="D5" s="20">
+        <v>11</v>
+      </c>
+      <c r="E5" s="21">
         <v>1500</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="19">
-        <f>D5*E5</f>
-        <v>12750</v>
+      <c r="G5" s="22">
+        <f t="shared" ref="G5:G6" si="0">D5*E5</f>
+        <v>16500</v>
       </c>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="6"/>
-      <c r="C6" s="20">
-        <v>46256</v>
-      </c>
-      <c r="D6" s="14">
-        <v>11</v>
-      </c>
-      <c r="E6" s="15">
+      <c r="C6" s="19">
+        <v>46257</v>
+      </c>
+      <c r="D6" s="20">
+        <v>6.75</v>
+      </c>
+      <c r="E6" s="21">
         <v>1500</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="21">
-        <f t="shared" ref="G6:G7" si="0">D6*E6</f>
-        <v>16500</v>
+      <c r="G6" s="22">
+        <f t="shared" si="0"/>
+        <v>10125</v>
       </c>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6"/>
-      <c r="C7" s="20">
-        <v>46257</v>
-      </c>
-      <c r="D7" s="14">
-        <v>6.75</v>
-      </c>
-      <c r="E7" s="15">
-        <v>1500</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" s="21">
-        <f t="shared" si="0"/>
-        <v>10125</v>
-      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="26"/>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="6"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="23"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8" s="30">
+        <f>SUM(G4:G6)</f>
+        <v>39375</v>
+      </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="23"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="34">
+        <f>G8*0.19</f>
+        <v>7481.25</v>
+      </c>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="23"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="35">
+        <f>G8+G9</f>
+        <v>46856.25</v>
+      </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="6"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="6"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="6"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="29" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="31">
-        <f>SUM(G5:G11)</f>
-        <v>39375</v>
-      </c>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="6"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="G14" s="35">
-        <f>G13*0.19</f>
-        <v>7481.25</v>
-      </c>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" s="36">
-        <f>G13+G14</f>
-        <v>46856.25</v>
-      </c>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="8"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="11"/>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="8"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Further improvement, framelines in Excel tables can be surpressed.
</commit_message>
<xml_diff>
--- a/data/rechnung/Rechnungsbeträge.xlsx
+++ b/data/rechnung/Rechnungsbeträge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frank\git\document-generator\data\rechnung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C649762E-30EA-490B-AE9B-4403274A6F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03ABE387-6C63-4F0F-9A6E-6BBEE39416A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40560" yWindow="4320" windowWidth="28800" windowHeight="15345" xr2:uid="{79AF68BE-ECC0-4E6F-85E2-599950CEF42A}"/>
   </bookViews>
@@ -389,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
@@ -417,7 +417,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -804,7 +803,7 @@
       </c>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="2:8" ht="27" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" ht="27.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6"/>
       <c r="C4" s="14">
         <v>46255</v>
@@ -813,18 +812,18 @@
         <v>8.5</v>
       </c>
       <c r="E4" s="16">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="18">
         <f>D4*E4</f>
-        <v>12750</v>
+        <v>850</v>
       </c>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6"/>
       <c r="C5" s="19">
         <v>46256</v>
@@ -832,15 +831,15 @@
       <c r="D5" s="20">
         <v>11</v>
       </c>
-      <c r="E5" s="21">
-        <v>1500</v>
+      <c r="E5" s="16">
+        <v>100</v>
       </c>
       <c r="F5" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="21">
         <f t="shared" ref="G5:G6" si="0">D5*E5</f>
-        <v>16500</v>
+        <v>1100</v>
       </c>
       <c r="H5" s="7"/>
     </row>
@@ -852,66 +851,66 @@
       <c r="D6" s="20">
         <v>6.75</v>
       </c>
-      <c r="E6" s="21">
-        <v>1500</v>
+      <c r="E6" s="16">
+        <v>100</v>
       </c>
       <c r="F6" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="21">
         <f t="shared" si="0"/>
-        <v>10125</v>
+        <v>675</v>
       </c>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="26"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="25"/>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="6"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="28" t="s">
+      <c r="C8" s="26"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="30">
+      <c r="G8" s="29">
         <f>SUM(G4:G6)</f>
-        <v>39375</v>
+        <v>2625</v>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="32" t="s">
+      <c r="C9" s="30"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="33">
         <f>G8*0.19</f>
-        <v>7481.25</v>
+        <v>498.75</v>
       </c>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="32" t="s">
+      <c r="C10" s="30"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="35">
+      <c r="G10" s="34">
         <f>G8+G9</f>
-        <v>46856.25</v>
+        <v>3123.75</v>
       </c>
       <c r="H10" s="7"/>
     </row>

</xml_diff>